<commit_message>
Riscrive le sequenze L4 come catene causali vere, non parole affiancate
Il primo giro (scheda "Sequenze (L4) - DRAFT") era 3 parole per fonema
senza un vero filo logico tra loro. Riscritte tutte e 25 come catena
causale/temporale reale (A porta a B, che porta a C), verificate contro
la frase che il gioco dice davvero ("Prima incontriamo... Poi arriva...
E infine ecco...") invece di restare solo tre figure affiancate. Aggiunta
una colonna che spiega il nesso causale di ciascuna, da rivedere prima di
entrare nel codice.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Torc6ixSdkF7HDXVqqw48E
</commit_message>
<xml_diff>
--- a/docs/Lallo_Catalogo_Contenuti.xlsx
+++ b/docs/Lallo_Catalogo_Contenuti.xlsx
@@ -38111,11 +38111,11 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -38131,27 +38131,27 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Parola 1 (Prima...)</t>
+          <t>Parola 1</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Parola 2 (Poi...)</t>
+          <t>Parola 2</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Parola 3 (E infine...)</t>
+          <t>Parola 3</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Frase d'esempio</t>
+          <t>Come si legge nel gioco</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>Nota / da validare</t>
+          <t>Perché ha senso (nesso causale/temporale)</t>
         </is>
       </c>
     </row>
@@ -38168,25 +38168,29 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>berretto</t>
+          <t>mucca</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>bicicletta</t>
+          <t>latte</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>bosco</t>
+          <t>burro</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Prima berretto, poi bicicletta, e infine bosco.</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr"/>
+          <t>Prima incontriamo mucca. Poi arriva latte. E infine ecco burro.</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>la mucca produce il latte, il latte lavorato diventa burro: filiera reale, in ordine.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -38201,25 +38205,29 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>cuoco</t>
+          <t>uovo</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>fuoco</t>
+          <t>oca</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>cucchiaio</t>
+          <t>acqua</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Prima cuoco, poi fuoco, e infine cucchiaio.</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr"/>
+          <t>Prima incontriamo uovo. Poi arriva oca. E infine ecco acqua.</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>dall'uovo nasce l'oca, che poi va a nuotare nell'acqua: ciclo di vita reale.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -38234,27 +38242,27 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>cena</t>
+          <t>farina</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>ciliegia</t>
+          <t>ciambella</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>ciambella</t>
+          <t>cioccolato</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Prima cena, poi ciliegia, e infine ciambella.</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>le 3 portate di una cena</t>
+          <t>Prima incontriamo farina. Poi arriva ciambella. E infine ecco cioccolato.</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>con la farina si fa l'impasto, si forma la ciambella, si guarnisce col cioccolato: passaggi di una vera ricetta.</t>
         </is>
       </c>
     </row>
@@ -38271,27 +38279,27 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>nido</t>
+          <t>farina</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>dinosauro</t>
+          <t>dolce</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>drago</t>
+          <t>candela</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Prima nido, poi dinosauro, e infine drago.</t>
-        </is>
-      </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>cornice fantastica, non biologica: nasce dal nido, cresce e "diventa" un drago leggendario — da confermare se va bene o va cambiata</t>
+          <t>Prima incontriamo farina. Poi arriva dolce. E infine ecco candela.</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>con la farina si fa il dolce, sul dolce finito si mette la candela: preparare una torta di compleanno, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38323,12 +38331,12 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Prima fiore, poi farfalla, e infine fragola.</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>fiore-impollinazione-frutto, come l'esempio del seme</t>
+          <t>Prima incontriamo fiore. Poi arriva farfalla. E infine ecco fragola.</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>il fiore attira la farfalla che lo impollina, e nasce la fragola: processo naturale reale (identico all'esempio seme→fiore→frutto).</t>
         </is>
       </c>
     </row>
@@ -38360,12 +38368,12 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Prima gomitolo, poi ago, e infine gonna.</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>lavoro a maglia: gomitolo di lana, ago, gonna cucita</t>
+          <t>Prima incontriamo gomitolo. Poi arriva ago. E infine ecco gonna.</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>dal gomitolo di lana, con l'ago, si cuce la gonna: i passaggi di un vero lavoro a maglia.</t>
         </is>
       </c>
     </row>
@@ -38387,22 +38395,22 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
+          <t>pioggia</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
           <t>girasole</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>raggio</t>
-        </is>
-      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Prima giardino, poi girasole, e infine raggio.</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>il girasole si gira verso il sole, come in natura</t>
+          <t>Prima incontriamo giardino. Poi arriva pioggia. E infine ecco girasole.</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>nel giardino arriva la pioggia, e grazie all'acqua cresce il girasole: causa→effetto reale.</t>
         </is>
       </c>
     </row>
@@ -38434,10 +38442,14 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Prima coniglio, poi foglia, e infine famiglia.</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr"/>
+          <t>Prima incontriamo coniglio. Poi arriva foglia. E infine ecco famiglia.</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>il coniglio trova una foglia, la mangia, poi torna dalla sua famiglia: una routine quotidiana in ordine.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -38452,27 +38464,27 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
+          <t>legno</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
           <t>ragno</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>ragnatela</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>bagno</t>
-        </is>
-      </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Prima ragno, poi ragnatela, e infine bagno.</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>scenetta comica: il ragno fa la tela in bagno</t>
+          <t>Prima incontriamo legno. Poi arriva ragno. E infine ecco ragnatela.</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>tra i rami di legno arriva il ragno, che tesse la ragnatela: cosa fanno davvero i ragni, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38504,12 +38516,12 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Prima sole, poi luna, e infine lampada.</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>giorno-notte-accendiamo la luce</t>
+          <t>Prima incontriamo sole. Poi arriva luna. E infine ecco lampada.</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>il sole tramonta, arriva la luna (è notte), e allora accendiamo la lampada: il ciclo giorno→notte reale.</t>
         </is>
       </c>
     </row>
@@ -38526,25 +38538,29 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>mamma</t>
+          <t>monte</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>merenda</t>
+          <t>mucca</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>mela</t>
+          <t>tramonto</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Prima mamma, poi merenda, e infine mela.</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr"/>
+          <t>Prima incontriamo monte. Poi arriva mucca. E infine ecco tramonto.</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>sul monte arriva la mucca a pascolare, pascola fino al tramonto: una giornata vera, in ordine.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -38559,25 +38575,29 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>notte</t>
+          <t>nuvola</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>nave</t>
+          <t>neve</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>nuvola</t>
+          <t>nido</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Prima notte, poi nave, e infine nuvola.</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr"/>
+          <t>Prima incontriamo nuvola. Poi arriva neve. E infine ecco nido.</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>dalla nuvola cade la neve, che copre il nido: causa→effetto meteo reale.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -38607,12 +38627,12 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Prima pianta, poi ombra, e infine vento.</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>crescita naturale: la pianta cresce, fa ombra, si muove col vento</t>
+          <t>Prima incontriamo pianta. Poi arriva ombra. E infine ecco vento.</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>la pianta cresce, fa ombra, e con il vento si muove: tre cose vere di una pianta, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38629,27 +38649,27 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>porta</t>
+          <t>nido</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>passero</t>
+          <t>uovo</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>pianoforte</t>
+          <t>pollo</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Prima porta, poi passero, e infine pianoforte.</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>scenetta: si apre la porta, entra un passero, si posa sul pianoforte</t>
+          <t>Prima incontriamo nido. Poi arriva uovo. E infine ecco pollo.</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>nel nido c'è l'uovo, dall'uovo nasce il pollo: lo stesso schema dell'esempio uovo→pulcino→pollo.</t>
         </is>
       </c>
     </row>
@@ -38671,22 +38691,22 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>rana</t>
+          <t>ramo</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>roccia</t>
+          <t>rosa</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Prima raggio, poi rana, e infine roccia.</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>il sole sveglia la rana che salta sulla roccia</t>
+          <t>Prima incontriamo raggio. Poi arriva ramo. E infine ecco rosa.</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>il raggio di sole scalda il ramo, e grazie al sole nasce la rosa: causa→effetto di una vera fioritura.</t>
         </is>
       </c>
     </row>
@@ -38718,12 +38738,12 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Prima prato, poi trifoglio, e infine bruco.</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>catena naturale nel prato</t>
+          <t>Prima incontriamo prato. Poi arriva trifoglio. E infine ecco bruco.</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>nel prato cresce il trifoglio, e arriva il bruco a mangiarlo: una vera catena naturale.</t>
         </is>
       </c>
     </row>
@@ -38755,12 +38775,12 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Prima orto, poi verdura, e infine torta.</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>dall'orto alla tavola</t>
+          <t>Prima incontriamo orto. Poi arriva verdura. E infine ecco torta.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>nell'orto cresce la verdura, che in cucina diventa una torta: dall'orto alla tavola, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38792,12 +38812,12 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Prima sole, poi sasso, e infine serpente.</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>il sole scalda il sasso, il serpente si scalda sopra</t>
+          <t>Prima incontriamo sole. Poi arriva sasso. E infine ecco serpente.</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>il sole scalda il sasso, e il serpente si scalda sopra: comportamento reale dei rettili, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38829,12 +38849,12 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Prima sveglia, poi vestito, e infine scuola.</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>routine del mattino</t>
+          <t>Prima incontriamo sveglia. Poi arriva vestito. E infine ecco scuola.</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>suona la sveglia, ci si veste, si va a scuola: la vera routine del mattino, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38866,12 +38886,12 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Prima guscio, poi nascita, e infine crescita.</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>il guscio si rompe, nasce, cresce — stesso schema "uovo-pulcino-pollo" ma con le parole SCI/SCE</t>
+          <t>Prima incontriamo guscio. Poi arriva nascita. E infine ecco crescita.</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>il guscio si rompe, c'è la nascita, poi la crescita: lo stesso schema di uovo→pulcino→pollo, con le parole SCI/SCE.</t>
         </is>
       </c>
     </row>
@@ -38903,12 +38923,12 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Prima gattino, poi gatto, e infine topo.</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>crescita dell'animale + comportamento (caccia)</t>
+          <t>Prima incontriamo gattino. Poi arriva gatto. E infine ecco topo.</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>il gattino cresce e diventa un gatto, che poi caccia il topo: crescita + conseguenza reale.</t>
         </is>
       </c>
     </row>
@@ -38940,12 +38960,12 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Prima vanga, poi ravanello, e infine vassoio.</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>dall'orto alla tavola, versione V</t>
+          <t>Prima incontriamo vanga. Poi arriva ravanello. E infine ecco vassoio.</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>con la vanga si scava, cresce il ravanello, si serve nel vassoio: dall'orto alla tavola, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38977,12 +38997,12 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Prima zolla, poi orzo, e infine pranzo.</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>dalla terra al pranzo</t>
+          <t>Prima incontriamo zolla. Poi arriva orzo. E infine ecco pranzo.</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>nella zolla di terra cresce l'orzo, pronto per il pranzo: dalla terra al piatto, in ordine.</t>
         </is>
       </c>
     </row>
@@ -39014,12 +39034,12 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Prima zolla, poi zucca, e infine zuppa.</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>dalla terra alla zuppa</t>
+          <t>Prima incontriamo zolla. Poi arriva zucca. E infine ecco zuppa.</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>nella zolla di terra cresce la zucca, che diventa una zuppa: dalla terra al piatto, in ordine.</t>
         </is>
       </c>
     </row>
@@ -39041,7 +39061,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>piazza</t>
+          <t>zucchero</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -39051,19 +39071,19 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Prima zucca, poi piazza, e infine zuppa.</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>dal mercato alla zuppa</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="70" customHeight="1">
+          <t>Prima incontriamo zucca. Poi arriva zucchero. E infine ecco zuppa.</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>la zucca matura, si aggiunge lo zucchero, diventa una zuppa dolce: i passaggi di una vera ricetta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="80" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Bozza mia, non ancora nel codice. Ogni riga usa parole già nel word bank del suo fonema quando possibile (stesse immagini/audio già pronti, nessun asset nuovo da generare) e punta a un filo logico reale (crescita, causa-effetto, routine quotidiana), sullo stesso modello di "seme→fiore→frutto" o "guscio→nascita→crescita". Correggi/sostituisci quello che non ti convince in questa stessa tabella: aggiorno il codice solo dopo la tua conferma.</t>
+          <t>Rifatta dopo il tuo feedback: la prima versione era 3 parole imparentate, non una storia. Ora ogni riga è una catena causale/temporale reale (A causa/porta a B, che porta a C), verificata leggendola con le frasi che il gioco usa davvero ("Prima incontriamo... Poi arriva... E infine ecco...", colonna F) — non solo tre figure affiancate. Correggi/sostituisci quello che non ti convince in questa stessa tabella: aggiorno il codice solo dopo la tua conferma.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sequenze L4: frammenti di frase causali al posto del connettore generico
Il connettore "Prima incontriamo.../Poi arriva.../E infine ecco..." era
identico per tutti i 25 fonemi: diceva l'ordine ma non il perché. Ogni
fonema ha ora il suo testo (Frammento 1/2/3) che spiega il nesso
causale attorno a ciascuna parola — la parola resta isolata e pronunciata
chiara a fine frammento (serve per l'allenamento del suono), ma il testo
intorno racconta la causa invece del semplice ordine. Aggiunta una
colonna "Frase completa" per sentire il risultato finale.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Torc6ixSdkF7HDXVqqw48E
</commit_message>
<xml_diff>
--- a/docs/Lallo_Catalogo_Contenuti.xlsx
+++ b/docs/Lallo_Catalogo_Contenuti.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Rime (L4)'!$A$1:$F$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Racconti (L4)'!$A$1:$G$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Giochi per livello'!$A$1:$E$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sequenze (L4) - DRAFT'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sequenze (L4) - DRAFT'!$A$1:$J$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38106,16 +38106,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="55" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -38131,25 +38134,40 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Frammento 1</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>Parola 1</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Frammento 2</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Parola 2</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Frammento 3</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Parola 3</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Come si legge nel gioco</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Frase completa</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Perché ha senso (nesso causale/temporale)</t>
         </is>
@@ -38168,25 +38186,40 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
+          <t>Ecco la</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
           <t>mucca</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>che dà il</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>latte</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>e diventa</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>burro</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo mucca. Poi arriva latte. E infine ecco burro.</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Ecco la mucca, che dà il latte, e diventa burro.</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>la mucca produce il latte, il latte lavorato diventa burro: filiera reale, in ordine.</t>
         </is>
@@ -38205,27 +38238,42 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
+          <t>Ecco l'</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
           <t>uovo</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>da cui nasce l'</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>oca</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>che va a nuotare nell'</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>acqua</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo uovo. Poi arriva oca. E infine ecco acqua.</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>dall'uovo nasce l'oca, che poi va a nuotare nell'acqua: ciclo di vita reale.</t>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Ecco l'uovo, da cui nasce l'oca, che va a nuotare nell'acqua.</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>dall'uovo nasce l'oca, che poi va a nuotare: ciclo di vita reale.</t>
         </is>
       </c>
     </row>
@@ -38242,27 +38290,42 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
+          <t>Con la</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
           <t>farina</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>si fa la</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>ciambella</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>e si guarnisce col</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>cioccolato</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo farina. Poi arriva ciambella. E infine ecco cioccolato.</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>con la farina si fa l'impasto, si forma la ciambella, si guarnisce col cioccolato: passaggi di una vera ricetta.</t>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Con la farina, si fa la ciambella, e si guarnisce col cioccolato.</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>con la farina si fa l'impasto, si forma la ciambella, si guarnisce col cioccolato: una vera ricetta, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38279,27 +38342,42 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
+          <t>Con la</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
           <t>farina</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>si fa un</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>dolce</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>e sopra mettiamo la</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>candela</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo farina. Poi arriva dolce. E infine ecco candela.</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>con la farina si fa il dolce, sul dolce finito si mette la candela: preparare una torta di compleanno, in ordine.</t>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Con la farina, si fa un dolce, e sopra mettiamo la candela.</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>con la farina si fa il dolce, sul dolce si mette la candela: una torta di compleanno, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38316,27 +38394,42 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
+          <t>Ecco il</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
           <t>fiore</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>che attira la</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>farfalla</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>e nasce la</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>fragola</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo fiore. Poi arriva farfalla. E infine ecco fragola.</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>il fiore attira la farfalla che lo impollina, e nasce la fragola: processo naturale reale (identico all'esempio seme→fiore→frutto).</t>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Ecco il fiore, che attira la farfalla, e nasce la fragola.</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>il fiore attira la farfalla che lo impollina, e nasce la fragola: processo naturale reale.</t>
         </is>
       </c>
     </row>
@@ -38353,25 +38446,40 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
+          <t>Dal</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
           <t>gomitolo</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>con l'</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>ago</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>si cuce la</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>gonna</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo gomitolo. Poi arriva ago. E infine ecco gonna.</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Dal gomitolo, con l'ago, si cuce la gonna.</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>dal gomitolo di lana, con l'ago, si cuce la gonna: i passaggi di un vero lavoro a maglia.</t>
         </is>
@@ -38390,25 +38498,40 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
+          <t>Nel</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
           <t>giardino</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>arriva la</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>pioggia</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>e cresce il</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>girasole</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo giardino. Poi arriva pioggia. E infine ecco girasole.</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Nel giardino, arriva la pioggia, e cresce il girasole.</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>nel giardino arriva la pioggia, e grazie all'acqua cresce il girasole: causa→effetto reale.</t>
         </is>
@@ -38427,27 +38550,42 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
+          <t>Ecco il</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
           <t>coniglio</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>che mangia una</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>foglia</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>e torna dalla</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>famiglia</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo coniglio. Poi arriva foglia. E infine ecco famiglia.</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>il coniglio trova una foglia, la mangia, poi torna dalla sua famiglia: una routine quotidiana in ordine.</t>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Ecco il coniglio, che mangia una foglia, e torna dalla famiglia.</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>il coniglio trova una foglia, la mangia, poi torna a casa: una routine quotidiana in ordine.</t>
         </is>
       </c>
     </row>
@@ -38464,27 +38602,42 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
+          <t>Tra i rami di</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
           <t>legno</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>arriva il</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>ragno</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>che tesse la</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>ragnatela</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo legno. Poi arriva ragno. E infine ecco ragnatela.</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>tra i rami di legno arriva il ragno, che tesse la ragnatela: cosa fanno davvero i ragni, in ordine.</t>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Tra i rami di legno, arriva il ragno, che tesse la ragnatela.</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>il ragno arriva tra i rami e tesse la sua ragnatela: cosa fanno davvero i ragni, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38501,27 +38654,42 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
+          <t>Tramonta il</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
           <t>sole</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>arriva la</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>luna</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>e accendiamo la</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>lampada</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo sole. Poi arriva luna. E infine ecco lampada.</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>il sole tramonta, arriva la luna (è notte), e allora accendiamo la lampada: il ciclo giorno→notte reale.</t>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Tramonta il sole, arriva la luna, e accendiamo la lampada.</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>il sole tramonta, arriva la notte, e allora accendiamo la luce: il ciclo giorno→notte reale.</t>
         </is>
       </c>
     </row>
@@ -38538,27 +38706,42 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
+          <t>Sul</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
           <t>monte</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>pascola la</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>mucca</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>fino al</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>tramonto</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo monte. Poi arriva mucca. E infine ecco tramonto.</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>sul monte arriva la mucca a pascolare, pascola fino al tramonto: una giornata vera, in ordine.</t>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Sul monte, pascola la mucca, fino al tramonto.</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>la mucca pascola sul monte fino a sera: una giornata vera, in ordine.</t>
         </is>
       </c>
     </row>
@@ -38575,25 +38758,40 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
+          <t>Dalla</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
           <t>nuvola</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>cade la</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>neve</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>che copre il</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>nido</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo nuvola. Poi arriva neve. E infine ecco nido.</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Dalla nuvola, cade la neve, che copre il nido.</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>dalla nuvola cade la neve, che copre il nido: causa→effetto meteo reale.</t>
         </is>
@@ -38612,25 +38810,40 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
+          <t>Cresce la</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
           <t>pianta</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>che fa</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>ombra</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>e si muove col</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>vento</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo pianta. Poi arriva ombra. E infine ecco vento.</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Cresce la pianta, che fa ombra, e si muove col vento.</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>la pianta cresce, fa ombra, e con il vento si muove: tre cose vere di una pianta, in ordine.</t>
         </is>
@@ -38649,27 +38862,42 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
+          <t>Nel</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
           <t>nido</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>c'è un</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>uovo</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>da cui nasce il</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>pollo</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo nido. Poi arriva uovo. E infine ecco pollo.</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>nel nido c'è l'uovo, dall'uovo nasce il pollo: lo stesso schema dell'esempio uovo→pulcino→pollo.</t>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Nel nido, c'è un uovo, da cui nasce il pollo.</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>nel nido c'è l'uovo, dall'uovo nasce il pollo: lo stesso schema di uovo→pulcino→pollo.</t>
         </is>
       </c>
     </row>
@@ -38686,25 +38914,40 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
+          <t>Il</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
           <t>raggio</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>scalda il</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>ramo</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>e fa sbocciare la</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>rosa</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo raggio. Poi arriva ramo. E infine ecco rosa.</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Il raggio, scalda il ramo, e fa sbocciare la rosa.</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>il raggio di sole scalda il ramo, e grazie al sole nasce la rosa: causa→effetto di una vera fioritura.</t>
         </is>
@@ -38723,25 +38966,40 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
+          <t>Nel</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
           <t>prato</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>cresce il</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>trifoglio</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>che mangia il</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>bruco</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo prato. Poi arriva trifoglio. E infine ecco bruco.</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Nel prato, cresce il trifoglio, che mangia il bruco.</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>nel prato cresce il trifoglio, e arriva il bruco a mangiarlo: una vera catena naturale.</t>
         </is>
@@ -38760,25 +39018,40 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
+          <t>Nell'</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
           <t>orto</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>cresce la</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>verdura</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>che diventa una</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>torta</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo orto. Poi arriva verdura. E infine ecco torta.</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Nell'orto, cresce la verdura, che diventa una torta.</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>nell'orto cresce la verdura, che in cucina diventa una torta: dall'orto alla tavola, in ordine.</t>
         </is>
@@ -38797,25 +39070,40 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
+          <t>Il</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
           <t>sole</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>scalda il</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>sasso</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>dove si scalda il</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>serpente</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo sole. Poi arriva sasso. E infine ecco serpente.</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Il sole, scalda il sasso, dove si scalda il serpente.</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>il sole scalda il sasso, e il serpente si scalda sopra: comportamento reale dei rettili, in ordine.</t>
         </is>
@@ -38834,25 +39122,40 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
+          <t>Suona la</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
           <t>sveglia</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>indossiamo il</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
         <is>
           <t>vestito</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>e andiamo a</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>scuola</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo sveglia. Poi arriva vestito. E infine ecco scuola.</t>
-        </is>
-      </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Suona la sveglia, indossiamo il vestito, e andiamo a scuola.</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>suona la sveglia, ci si veste, si va a scuola: la vera routine del mattino, in ordine.</t>
         </is>
@@ -38871,25 +39174,40 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
+          <t>Si rompe il</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
           <t>guscio</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>c'è la</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>nascita</t>
         </is>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>e poi la</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>crescita</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo guscio. Poi arriva nascita. E infine ecco crescita.</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Si rompe il guscio, c'è la nascita, e poi la crescita.</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>il guscio si rompe, c'è la nascita, poi la crescita: lo stesso schema di uovo→pulcino→pollo, con le parole SCI/SCE.</t>
         </is>
@@ -38908,25 +39226,40 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
+          <t>Il</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
           <t>gattino</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>cresce e diventa un</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>gatto</t>
         </is>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>che caccia il</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>topo</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo gattino. Poi arriva gatto. E infine ecco topo.</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Il gattino, cresce e diventa un gatto, che caccia il topo.</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>il gattino cresce e diventa un gatto, che poi caccia il topo: crescita + conseguenza reale.</t>
         </is>
@@ -38945,25 +39278,40 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
+          <t>Con la</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
           <t>vanga</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>si scava, cresce il</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>ravanello</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>e si serve nel</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>vassoio</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo vanga. Poi arriva ravanello. E infine ecco vassoio.</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Con la vanga, si scava, cresce il ravanello, e si serve nel vassoio.</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>con la vanga si scava, cresce il ravanello, si serve nel vassoio: dall'orto alla tavola, in ordine.</t>
         </is>
@@ -38982,25 +39330,40 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
+          <t>Nella</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
           <t>zolla</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>cresce l'</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>orzo</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>pronto per il</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>pranzo</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo zolla. Poi arriva orzo. E infine ecco pranzo.</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Nella zolla, cresce l'orzo, pronto per il pranzo.</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
         <is>
           <t>nella zolla di terra cresce l'orzo, pronto per il pranzo: dalla terra al piatto, in ordine.</t>
         </is>
@@ -39019,25 +39382,40 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
+          <t>Nella</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
           <t>zolla</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>cresce la</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>zucca</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>che diventa una</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>zuppa</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo zolla. Poi arriva zucca. E infine ecco zuppa.</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Nella zolla, cresce la zucca, che diventa una zuppa.</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>nella zolla di terra cresce la zucca, che diventa una zuppa: dalla terra al piatto, in ordine.</t>
         </is>
@@ -39056,41 +39434,56 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
+          <t>Matura la</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
           <t>zucca</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>si aggiunge lo</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>zucchero</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>diventa una</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>zuppa</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Prima incontriamo zucca. Poi arriva zucchero. E infine ecco zuppa.</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Matura la zucca, si aggiunge lo zucchero, diventa una zuppa.</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>la zucca matura, si aggiunge lo zucchero, diventa una zuppa dolce: i passaggi di una vera ricetta.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="80" customHeight="1">
+    <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rifatta dopo il tuo feedback: la prima versione era 3 parole imparentate, non una storia. Ora ogni riga è una catena causale/temporale reale (A causa/porta a B, che porta a C), verificata leggendola con le frasi che il gioco usa davvero ("Prima incontriamo... Poi arriva... E infine ecco...", colonna F) — non solo tre figure affiancate. Correggi/sostituisci quello che non ti convince in questa stessa tabella: aggiorno il codice solo dopo la tua conferma.</t>
+          <t>Rifatta di nuovo dopo il tuo feedback: via il connettore generico "Prima incontriamo.../Poi arriva.../E infine ecco..." uguale per tutti i fonemi, ora ogni fonema ha il SUO testo che spiega perché una cosa porta all'altra (colonne Frammento 1/2/3, una parte di frase per ogni immagine) — la parola resta comunque isolata e pronunciata chiara alla fine di ogni frammento (serve per l'allenamento del suono), ma il testo intorno ora racconta la causa, non solo l'ordine. Colonna "Frase completa" per sentire il risultato finale, colonna "Perché ha senso" per il nesso dietro ogni scelta. Correggi/sostituisci quello che non ti convince in questa stessa tabella: aggiorno il codice solo dopo la tua conferma.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:J26"/>
   <mergeCells count="1">
-    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A28:J28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sequenze L4: applica le correzioni del founder, segnala le 7 parole nuove
Applicate le correzioni dirette sulle 25 frasi (Teo il gatto, zio nel
giardino, api->ape/topi->topo/ravanelli->ravanello per riusare l'audio
già pronto, Halloween mantenuto con una nuova parola "lanterna" invece
di "zuppa"). Aggiunta una colonna Stato: 7 parole non hanno ancora
illustrazione+audio (collina, pollaio, pulcino, roseto, minestrone,
gheriglio, lanterna) — generazione in corso con lo stesso stile/voce
del resto del word bank.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Torc6ixSdkF7HDXVqqw48E
</commit_message>
<xml_diff>
--- a/docs/Lallo_Catalogo_Contenuti.xlsx
+++ b/docs/Lallo_Catalogo_Contenuti.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Rime (L4)'!$A$1:$F$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Racconti (L4)'!$A$1:$G$101</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Giochi per livello'!$A$1:$E$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sequenze (L4) - DRAFT'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Sequenze (L4) - DRAFT'!$A$1:$K$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -118,6 +118,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -38106,19 +38109,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -38134,1340 +38138,1470 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
+          <t>Stato</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
           <t>Frammento 1</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Parola 1</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Frammento 2</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Parola 2</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Frammento 3</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Parola 3</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Frase completa</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Perché ha senso (nesso causale/temporale)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>Ecco la</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>mucca</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="F2" s="10" t="inlineStr">
         <is>
           <t>che dà il</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="G2" s="10" t="inlineStr">
         <is>
           <t>latte</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>e diventa</t>
-        </is>
-      </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>che poi diventa</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="inlineStr">
         <is>
           <t>burro</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>Ecco la mucca, che dà il latte, e diventa burro.</t>
-        </is>
-      </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>Ecco la mucca, che dà il latte, che poi diventa burro.</t>
+        </is>
+      </c>
+      <c r="K2" s="10" t="inlineStr">
         <is>
           <t>la mucca produce il latte, il latte lavorato diventa burro: filiera reale, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>C (dura)</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Ecco l'</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>uovo</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
         <is>
           <t>da cui nasce l'</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>oca</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>che va a nuotare nell'</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>acqua</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>Ecco l'uovo, da cui nasce l'oca, che va a nuotare nell'acqua.</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>dall'uovo nasce l'oca, che poi va a nuotare: ciclo di vita reale.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>CI (dolce)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>ci</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Con la</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>farina</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>si fa la</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>prepariamo una</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
         <is>
           <t>ciambella</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>e si guarnisce col</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>che si guarnisce col</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
         <is>
           <t>cioccolato</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Con la farina, si fa la ciambella, e si guarnisce col cioccolato.</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Con la farina, prepariamo una ciambella, che si guarnisce col cioccolato.</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
         <is>
           <t>con la farina si fa l'impasto, si forma la ciambella, si guarnisce col cioccolato: una vera ricetta, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Con la</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>farina</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>si fa un</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>prepariamo un</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>dolce</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>e sopra mettiamo la</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr">
-        <is>
-          <t>candela</t>
-        </is>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>Con la farina, si fa un dolce, e sopra mettiamo la candela.</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>con la farina si fa il dolce, sul dolce si mette la candela: una torta di compleanno, in ordine.</t>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>da portare in dono alla</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>nonna</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>Con la farina, prepariamo un dolce, da portare in dono alla nonna.</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>con la farina si fa il dolce, il dolce si regala alla nonna: una vera occasione (es. una visita), in ordine.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>f</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Ecco il</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>fiore</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>che attira la</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="G6" s="10" t="inlineStr">
         <is>
           <t>farfalla</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>e nasce la</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>fragola</t>
-        </is>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Ecco il fiore, che attira la farfalla, e nasce la fragola.</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr">
-        <is>
-          <t>il fiore attira la farfalla che lo impollina, e nasce la fragola: processo naturale reale.</t>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>e poi arriva l'</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>ape</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>Ecco il fiore, che attira la farfalla, e poi arriva l'ape.</t>
+        </is>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>il fiore attira prima la farfalla e poi l'ape, entrambe impollinatrici: comportamento naturale reale, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>G (dura)</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Dal</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>gomitolo</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>con l'</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
         <is>
           <t>ago</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>si cuce la</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>gonna</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="J7" s="10" t="inlineStr">
         <is>
           <t>Dal gomitolo, con l'ago, si cuce la gonna.</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>dal gomitolo di lana, con l'ago, si cuce la gonna: i passaggi di un vero lavoro a maglia.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>GI (dolce)</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>gi</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Nel</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>giardino</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
         <is>
           <t>arriva la</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>pioggia</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>e cresce il</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>girasole</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>Nel giardino, arriva la pioggia, e cresce il girasole.</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>nel giardino arriva la pioggia, e grazie all'acqua cresce il girasole: causa→effetto reale.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>GLI</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>gli</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Ecco il</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>coniglio</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>che mangia una</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>foglia</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>e torna dalla</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>famiglia</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Ecco il coniglio, che mangia una foglia, e torna dalla famiglia.</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>il coniglio trova una foglia, la mangia, poi torna a casa: una routine quotidiana in ordine.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>GN</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>gn</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Tra i rami di</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>legno</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="F10" s="10" t="inlineStr">
         <is>
           <t>arriva il</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="G10" s="10" t="inlineStr">
         <is>
           <t>ragno</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>che tesse la</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>ragnatela</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>Tra i rami di legno, arriva il ragno, che tesse la ragnatela.</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>il ragno arriva tra i rami e tesse la sua ragnatela: cosa fanno davvero i ragni, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>l</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Tramonta il</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>sole</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="F11" s="10" t="inlineStr">
         <is>
           <t>arriva la</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
         <is>
           <t>luna</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>e accendiamo la</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>lampada</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>Tramonta il sole, arriva la luna, e accendiamo la lampada.</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>il sole tramonta, arriva la notte, e allora accendiamo la luce: il ciclo giorno→notte reale.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Sul</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>monte</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="F12" s="10" t="inlineStr">
         <is>
           <t>pascola la</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>mucca</t>
         </is>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>fino al</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>tramonto</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr">
         <is>
           <t>Sul monte, pascola la mucca, fino al tramonto.</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>la mucca pascola sul monte fino a sera: una giornata vera, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Dalla</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>nuvola</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>cade la</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>neve</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>che copre il</t>
-        </is>
-      </c>
-      <c r="H13" s="8" t="inlineStr">
-        <is>
-          <t>nido</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr">
-        <is>
-          <t>Dalla nuvola, cade la neve, che copre il nido.</t>
-        </is>
-      </c>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>dalla nuvola cade la neve, che copre il nido: causa→effetto meteo reale.</t>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>che copre la</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>collina</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="inlineStr">
+        <is>
+          <t>Dalla nuvola, cade la neve, che copre la collina.</t>
+        </is>
+      </c>
+      <c r="K13" s="9" t="inlineStr">
+        <is>
+          <t>dalla nuvola cade la neve, che copre la collina: causa→effetto meteo reale.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>M/N/L + cons.</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>mnl_cons</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Cresce la</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>pianta</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="F14" s="10" t="inlineStr">
         <is>
           <t>che fa</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="G14" s="10" t="inlineStr">
         <is>
           <t>ombra</t>
         </is>
       </c>
-      <c r="G14" s="8" t="inlineStr">
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>e si muove col</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>vento</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="J14" s="10" t="inlineStr">
         <is>
           <t>Cresce la pianta, che fa ombra, e si muove col vento.</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="K14" s="10" t="inlineStr">
         <is>
           <t>la pianta cresce, fa ombra, e con il vento si muove: tre cose vere di una pianta, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Nel</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>nido</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>pollaio</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>c'è un</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>uovo</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>da cui nasce il</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
-        <is>
-          <t>pollo</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Nel nido, c'è un uovo, da cui nasce il pollo.</t>
-        </is>
-      </c>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>nel nido c'è l'uovo, dall'uovo nasce il pollo: lo stesso schema di uovo→pulcino→pollo.</t>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>pulcino</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>Nel pollaio, c'è un uovo, da cui nasce il pulcino.</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>nel pollaio c'è l'uovo, dall'uovo nasce il pulcino: lo schema uovo→pulcino→pollo, versione completa.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>r</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Il</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>raggio</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>scalda il</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>ramo</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>roseto</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>e fa sbocciare la</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="I16" s="9" t="inlineStr">
         <is>
           <t>rosa</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>Il raggio, scalda il ramo, e fa sbocciare la rosa.</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>il raggio di sole scalda il ramo, e grazie al sole nasce la rosa: causa→effetto di una vera fioritura.</t>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>Il raggio, scalda il roseto, e fa sbocciare la rosa.</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>il raggio di sole scalda il roseto, e grazie al sole nasce la rosa: causa→effetto di una vera fioritura.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>cons. + R</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>cons_r</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>Nel</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>prato</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>cresce il</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
         <is>
           <t>trifoglio</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>che mangia il</t>
-        </is>
-      </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>che sfama il</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>bruco</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>Nel prato, cresce il trifoglio, che mangia il bruco.</t>
-        </is>
-      </c>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>nel prato cresce il trifoglio, e arriva il bruco a mangiarlo: una vera catena naturale.</t>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>Nel prato, cresce il trifoglio, che sfama il bruco.</t>
+        </is>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>nel prato cresce il trifoglio, che sfama il bruco: una vera catena naturale.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>R + cons.</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>r_cons</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Nell'</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>orto</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>cresce la</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>verdura</t>
         </is>
       </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>che diventa una</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
-        <is>
-          <t>torta</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Nell'orto, cresce la verdura, che diventa una torta.</t>
-        </is>
-      </c>
-      <c r="J18" s="8" t="inlineStr">
-        <is>
-          <t>nell'orto cresce la verdura, che in cucina diventa una torta: dall'orto alla tavola, in ordine.</t>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>che diventerà un</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>minestrone</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>Nell'orto, cresce la verdura, che diventerà un minestrone.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>nell'orto cresce la verdura, che in cucina diventa un minestrone: dall'orto alla tavola, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>Il</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>sole</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
         <is>
           <t>scalda il</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>sasso</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>dove si scalda il</t>
-        </is>
-      </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>dove si stende il</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>serpente</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>Il sole, scalda il sasso, dove si scalda il serpente.</t>
-        </is>
-      </c>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>il sole scalda il sasso, e il serpente si scalda sopra: comportamento reale dei rettili, in ordine.</t>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>Il sole, scalda il sasso, dove si stende il serpente.</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>il sole scalda il sasso, e il serpente si stende sopra: comportamento reale dei rettili, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>S + cons.</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>s_cons</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>Suona la</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>sveglia</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>indossiamo il</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>vestito</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>e andiamo a</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>scuola</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="J20" s="10" t="inlineStr">
         <is>
           <t>Suona la sveglia, indossiamo il vestito, e andiamo a scuola.</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="K20" s="10" t="inlineStr">
         <is>
           <t>suona la sveglia, ci si veste, si va a scuola: la vera routine del mattino, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>SCI/SCE</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>sci_sce</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Si rompe il</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>guscio</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>c'è la</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>nascita</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>e poi la</t>
-        </is>
-      </c>
-      <c r="H21" s="8" t="inlineStr">
-        <is>
-          <t>crescita</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Si rompe il guscio, c'è la nascita, e poi la crescita.</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>il guscio si rompe, c'è la nascita, poi la crescita: lo stesso schema di uovo→pulcino→pollo, con le parole SCI/SCE.</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Si rompe il guscio della</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>noce</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>esce il</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>gheriglio</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>che poi mangia lo</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>scoiattolo</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>Si rompe il guscio della noce, esce il gheriglio, che poi mangia lo scoiattolo.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>il guscio della noce si rompe, esce il gheriglio, che lo scoiattolo mangia: una vera catena naturale.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Il</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>gattino</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>cresce e diventa un</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>Ecco il</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>gatto</t>
         </is>
       </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>che caccia il</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>che si chiama Teo e salta sul</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>tetto</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>per cacciare il</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>topo</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>Il gattino, cresce e diventa un gatto, che caccia il topo.</t>
-        </is>
-      </c>
-      <c r="J22" s="8" t="inlineStr">
-        <is>
-          <t>il gattino cresce e diventa un gatto, che poi caccia il topo: crescita + conseguenza reale.</t>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>Ecco il gatto, che si chiama Teo e salta sul tetto, per cacciare il topo.</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>il gatto Teo sale sul tetto per cacciare il topo: un'azione reale, in ordine (il nome è solo un dettaglio, come "Rocco il robot" in Racconta la storia).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>v</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>Con la</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>vanga</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>si scava, cresce il</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>raccogliamo il</t>
+        </is>
+      </c>
+      <c r="G23" s="10" t="inlineStr">
         <is>
           <t>ravanello</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>e si serve nel</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>che disponiamo in un</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>vassoio</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>Con la vanga, si scava, cresce il ravanello, e si serve nel vassoio.</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>con la vanga si scava, cresce il ravanello, si serve nel vassoio: dall'orto alla tavola, in ordine.</t>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>Con la vanga, raccogliamo il ravanello, che disponiamo in un vassoio.</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>con la vanga si raccoglie il ravanello, che si serve nel vassoio: dall'orto alla tavola, in ordine.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Z (sonora, dz)</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>z_dz</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>Ecco lo</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>zio</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>nel suo giardino coltiva l'</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>orzo</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>che cuciniamo per il</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>pranzo</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>Ecco lo zio, nel suo giardino coltiva l'orzo, che cuciniamo per il pranzo.</t>
+        </is>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>lo zio coltiva l'orzo nel suo giardino, che diventa il pranzo: dalla coltivazione al piatto, in ordine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Zeta</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>zeta</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>In generazione (nuova illustrazione+audio)</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Nella</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>zolla</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>cresce l'</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>orzo</t>
-        </is>
-      </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>pronto per il</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>pranzo</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Nella zolla, cresce l'orzo, pronto per il pranzo.</t>
-        </is>
-      </c>
-      <c r="J24" s="8" t="inlineStr">
-        <is>
-          <t>nella zolla di terra cresce l'orzo, pronto per il pranzo: dalla terra al piatto, in ordine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Zeta</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>zeta</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Nella</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>zolla</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>cresce la</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>zucca</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>che diventa una</t>
-        </is>
-      </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>che a Halloween intagliamo in una</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>lanterna</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>Nella zolla, cresce la zucca, che a Halloween intagliamo in una lanterna.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>la zucca cresce dalla terra, e a Halloween si intaglia in una lanterna: un vero uso stagionale, in ordine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Z (sorda, ts)</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>z_ts</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (parole già illustrate)</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>Matura la</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>zucca</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>si aggiunge lo</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>zucchero</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>e si prepara la</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
         <is>
           <t>zuppa</t>
         </is>
       </c>
-      <c r="I25" s="8" t="inlineStr">
-        <is>
-          <t>Nella zolla, cresce la zucca, che diventa una zuppa.</t>
-        </is>
-      </c>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>nella zolla di terra cresce la zucca, che diventa una zuppa: dalla terra al piatto, in ordine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Z (sorda, ts)</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>z_ts</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Matura la</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>zucca</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>si aggiunge lo</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>zucchero</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>diventa una</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>zuppa</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>Matura la zucca, si aggiunge lo zucchero, diventa una zuppa.</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>Matura la zucca, si aggiunge lo zucchero, e si prepara la zuppa.</t>
+        </is>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
         <is>
           <t>la zucca matura, si aggiunge lo zucchero, diventa una zuppa dolce: i passaggi di una vera ricetta.</t>
         </is>
@@ -39476,14 +39610,14 @@
     <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Rifatta di nuovo dopo il tuo feedback: via il connettore generico "Prima incontriamo.../Poi arriva.../E infine ecco..." uguale per tutti i fonemi, ora ogni fonema ha il SUO testo che spiega perché una cosa porta all'altra (colonne Frammento 1/2/3, una parte di frase per ogni immagine) — la parola resta comunque isolata e pronunciata chiara alla fine di ogni frammento (serve per l'allenamento del suono), ma il testo intorno ora racconta la causa, non solo l'ordine. Colonna "Frase completa" per sentire il risultato finale, colonna "Perché ha senso" per il nesso dietro ogni scelta. Correggi/sostituisci quello che non ti convince in questa stessa tabella: aggiorno il codice solo dopo la tua conferma.</t>
+          <t>Versione con le tue correzioni applicate. Verde = pronta subito (usa solo parole già illustrate/con audio). Giallo = in generazione: la frase usa una parola nuova (collina, pollaio, pulcino, roseto, minestrone, gheriglio, lanterna) — sto creando illustrazione+audio nello stesso stile/voce di tutto il resto, aggiorno questa colonna quando sono pronte. "Teo" (T) resta come nome proprio dentro il testo parlato, zero lavoro extra, stesso schema di "Rocco il robot" in Racconta la storia. Per Z (sorda, ts) ho sostituito "cucina" con "zucchero" (un ambiente non si illustra bene come un singolo oggetto, un ingrediente sì) — dimmi se preferisci che generi comunque "cucina".</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:K26"/>
   <mergeCells count="1">
-    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A28:K28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Segna le 25 Sequenze illustrate come pronte nel catalogo
Le 7 illustrazioni (caricate dal founder) e i relativi audio (generati
in questa sessione) sono completi e già nel codice — aggiorna lo stato
da "in generazione" a "pronta" per tutte le righe.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Torc6ixSdkF7HDXVqqw48E
</commit_message>
<xml_diff>
--- a/docs/Lallo_Catalogo_Contenuti.xlsx
+++ b/docs/Lallo_Catalogo_Contenuti.xlsx
@@ -38810,57 +38810,57 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Dalla</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>nuvola</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="10" t="inlineStr">
         <is>
           <t>cade la</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
         <is>
           <t>neve</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>che copre la</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>collina</t>
         </is>
       </c>
-      <c r="J13" s="9" t="inlineStr">
+      <c r="J13" s="10" t="inlineStr">
         <is>
           <t>Dalla nuvola, cade la neve, che copre la collina.</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>dalla nuvola cade la neve, che copre la collina: causa→effetto meteo reale.</t>
         </is>
@@ -38924,114 +38924,114 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>Nel</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>pollaio</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>c'è un</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>uovo</t>
         </is>
       </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>da cui nasce il</t>
         </is>
       </c>
-      <c r="I15" s="9" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>pulcino</t>
         </is>
       </c>
-      <c r="J15" s="9" t="inlineStr">
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>Nel pollaio, c'è un uovo, da cui nasce il pulcino.</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>nel pollaio c'è l'uovo, dall'uovo nasce il pulcino: lo schema uovo→pulcino→pollo, versione completa.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>r</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>Il</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>raggio</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>scalda il</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>roseto</t>
         </is>
       </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>e fa sbocciare la</t>
         </is>
       </c>
-      <c r="I16" s="9" t="inlineStr">
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>rosa</t>
         </is>
       </c>
-      <c r="J16" s="9" t="inlineStr">
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>Il raggio, scalda il roseto, e fa sbocciare la rosa.</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>il raggio di sole scalda il roseto, e grazie al sole nasce la rosa: causa→effetto di una vera fioritura.</t>
         </is>
@@ -39095,57 +39095,57 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>R + cons.</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>r_cons</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>Nell'</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>orto</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>cresce la</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G18" s="10" t="inlineStr">
         <is>
           <t>verdura</t>
         </is>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>che diventerà un</t>
         </is>
       </c>
-      <c r="I18" s="9" t="inlineStr">
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>minestrone</t>
         </is>
       </c>
-      <c r="J18" s="9" t="inlineStr">
+      <c r="J18" s="10" t="inlineStr">
         <is>
           <t>Nell'orto, cresce la verdura, che diventerà un minestrone.</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>nell'orto cresce la verdura, che in cucina diventa un minestrone: dall'orto alla tavola, in ordine.</t>
         </is>
@@ -39266,57 +39266,57 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>SCI/SCE</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>sci_sce</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
         <is>
           <t>Si rompe il guscio della</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>noce</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>esce il</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>gheriglio</t>
         </is>
       </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>che poi mangia lo</t>
         </is>
       </c>
-      <c r="I21" s="9" t="inlineStr">
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>scoiattolo</t>
         </is>
       </c>
-      <c r="J21" s="9" t="inlineStr">
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>Si rompe il guscio della noce, esce il gheriglio, che poi mangia lo scoiattolo.</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="K21" s="10" t="inlineStr">
         <is>
           <t>il guscio della noce si rompe, esce il gheriglio, che lo scoiattolo mangia: una vera catena naturale.</t>
         </is>
@@ -39494,57 +39494,57 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Zeta</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>zeta</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>In generazione (nuova illustrazione+audio)</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Pronta (illustrazione+audio completati)</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
         <is>
           <t>Nella</t>
         </is>
       </c>
-      <c r="E25" s="9" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>zolla</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>cresce la</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>zucca</t>
         </is>
       </c>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="H25" s="10" t="inlineStr">
         <is>
           <t>che a Halloween intagliamo in una</t>
         </is>
       </c>
-      <c r="I25" s="9" t="inlineStr">
+      <c r="I25" s="10" t="inlineStr">
         <is>
           <t>lanterna</t>
         </is>
       </c>
-      <c r="J25" s="9" t="inlineStr">
+      <c r="J25" s="10" t="inlineStr">
         <is>
           <t>Nella zolla, cresce la zucca, che a Halloween intagliamo in una lanterna.</t>
         </is>
       </c>
-      <c r="K25" s="9" t="inlineStr">
+      <c r="K25" s="10" t="inlineStr">
         <is>
           <t>la zucca cresce dalla terra, e a Halloween si intaglia in una lanterna: un vero uso stagionale, in ordine.</t>
         </is>

</xml_diff>